<commit_message>
Acotar edificios de una cubicacion
</commit_message>
<xml_diff>
--- a/tests/fixtures/cubicacion-alcance-76-77.xlsx
+++ b/tests/fixtures/cubicacion-alcance-76-77.xlsx
@@ -3,7 +3,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>CUBICACION Nº8 - EDIFICIOS 76 Y 77</t>
   </si>
@@ -12,6 +12,30 @@
   </si>
   <si>
     <t>% Avance fisico ejecutado</t>
+  </si>
+  <si>
+    <t>Inventario historico de apartamentos</t>
+  </si>
+  <si>
+    <t>TH-01</t>
+  </si>
+  <si>
+    <t>TH-07</t>
+  </si>
+  <si>
+    <t>TH-19</t>
+  </si>
+  <si>
+    <t>TH-31</t>
+  </si>
+  <si>
+    <t>TH-53</t>
+  </si>
+  <si>
+    <t>TH-69</t>
+  </si>
+  <si>
+    <t>TH-73</t>
   </si>
 </sst>
 </file>
@@ -37,6 +61,34 @@
         <v>0.1845</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>